<commit_message>
feat: ajouter le champ financement et adapter les formulaires pour la gestion des lots mixtes en conventions foyer-résidence
</commit_message>
<xml_diff>
--- a/static/files/foyer_residence_logements.xlsx
+++ b/static/files/foyer_residence_logements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicolasoudard/workspace/beta.gouv.fr/apilos/static/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayoub.bouchachia\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD775BD-7784-D74C-BFAA-AB9A8474BCD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C234B24-6EDA-400B-B94E-576E934924E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36340" yWindow="2120" windowWidth="27400" windowHeight="16440" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
+    <workbookView xWindow="2655" yWindow="2595" windowWidth="21600" windowHeight="11295" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Logements" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Ici quelques explications</t>
   </si>
@@ -113,6 +113,9 @@
   </si>
   <si>
     <t>T1 bis</t>
+  </si>
+  <si>
+    <t>Financement</t>
   </si>
 </sst>
 </file>
@@ -339,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -370,6 +373,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -475,7 +484,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -771,354 +780,398 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08021C90-1ACF-2A4C-A1B0-58A48A8F7007}">
-  <dimension ref="A1:L51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
-    <col min="2" max="4" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="29.625" customWidth="1"/>
+    <col min="2" max="4" width="20.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="E1" s="22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="23"/>
-    </row>
-    <row r="3" spans="1:12" ht="19" x14ac:dyDescent="0.25">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="23"/>
+    </row>
+    <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="11"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="14" t="s">
+      <c r="D3" s="11"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="7"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="16"/>
-      <c r="E4" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="16"/>
+      <c r="F4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="9"/>
       <c r="C5" s="11"/>
-      <c r="D5" s="15"/>
-    </row>
-    <row r="6" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="11"/>
+      <c r="E5" s="15"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="7"/>
       <c r="C6" s="12"/>
-      <c r="D6" s="16"/>
-    </row>
-    <row r="7" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="12"/>
+      <c r="E6" s="16"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
       <c r="B7" s="9"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="4"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="15"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="7"/>
       <c r="C8" s="12"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="4"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-    </row>
-    <row r="9" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="11"/>
-      <c r="D9" s="15"/>
-    </row>
-    <row r="10" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="11"/>
+      <c r="E9" s="15"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="7"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="16"/>
-    </row>
-    <row r="11" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="12"/>
+      <c r="E10" s="16"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="9"/>
       <c r="C11" s="11"/>
-      <c r="D11" s="15"/>
-    </row>
-    <row r="12" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="11"/>
+      <c r="E11" s="15"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="12"/>
+      <c r="E12" s="16"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="9"/>
       <c r="C13" s="11"/>
-      <c r="D13" s="15"/>
-    </row>
-    <row r="14" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="11"/>
+      <c r="E13" s="15"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="7"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="16"/>
-    </row>
-    <row r="15" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D14" s="12"/>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="9"/>
       <c r="C15" s="11"/>
-      <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D15" s="11"/>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
       <c r="B16" s="7"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="16"/>
-    </row>
-    <row r="17" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D16" s="12"/>
+      <c r="E16" s="16"/>
+    </row>
+    <row r="17" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="9"/>
       <c r="C17" s="11"/>
-      <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="11"/>
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
       <c r="B18" s="7"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="16"/>
-    </row>
-    <row r="19" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D18" s="12"/>
+      <c r="E18" s="16"/>
+    </row>
+    <row r="19" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
       <c r="B19" s="9"/>
       <c r="C19" s="11"/>
-      <c r="D19" s="15"/>
-    </row>
-    <row r="20" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D19" s="11"/>
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
       <c r="B20" s="7"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="16"/>
-    </row>
-    <row r="21" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D20" s="12"/>
+      <c r="E20" s="16"/>
+    </row>
+    <row r="21" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="9"/>
       <c r="C21" s="11"/>
-      <c r="D21" s="15"/>
-    </row>
-    <row r="22" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D21" s="11"/>
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
       <c r="B22" s="7"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="16"/>
-    </row>
-    <row r="23" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D22" s="12"/>
+      <c r="E22" s="16"/>
+    </row>
+    <row r="23" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="9"/>
       <c r="C23" s="11"/>
-      <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D23" s="11"/>
+      <c r="E23" s="15"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="7"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="16"/>
-    </row>
-    <row r="25" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D24" s="12"/>
+      <c r="E24" s="16"/>
+    </row>
+    <row r="25" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
       <c r="B25" s="9"/>
       <c r="C25" s="11"/>
-      <c r="D25" s="15"/>
-    </row>
-    <row r="26" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="11"/>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="7"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="16"/>
-    </row>
-    <row r="27" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D26" s="12"/>
+      <c r="E26" s="16"/>
+    </row>
+    <row r="27" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8"/>
       <c r="B27" s="9"/>
       <c r="C27" s="11"/>
-      <c r="D27" s="15"/>
-    </row>
-    <row r="28" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D27" s="11"/>
+      <c r="E27" s="15"/>
+    </row>
+    <row r="28" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="7"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="16"/>
-    </row>
-    <row r="29" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D28" s="12"/>
+      <c r="E28" s="16"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
       <c r="B29" s="9"/>
       <c r="C29" s="11"/>
-      <c r="D29" s="15"/>
-    </row>
-    <row r="30" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D29" s="11"/>
+      <c r="E29" s="15"/>
+    </row>
+    <row r="30" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="7"/>
       <c r="C30" s="12"/>
-      <c r="D30" s="16"/>
-    </row>
-    <row r="31" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D30" s="12"/>
+      <c r="E30" s="16"/>
+    </row>
+    <row r="31" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
       <c r="B31" s="9"/>
       <c r="C31" s="11"/>
-      <c r="D31" s="15"/>
-    </row>
-    <row r="32" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D31" s="11"/>
+      <c r="E31" s="15"/>
+    </row>
+    <row r="32" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="7"/>
       <c r="C32" s="12"/>
-      <c r="D32" s="16"/>
-    </row>
-    <row r="33" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D32" s="12"/>
+      <c r="E32" s="16"/>
+    </row>
+    <row r="33" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
       <c r="B33" s="9"/>
       <c r="C33" s="11"/>
-      <c r="D33" s="15"/>
-    </row>
-    <row r="34" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D33" s="11"/>
+      <c r="E33" s="15"/>
+    </row>
+    <row r="34" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
       <c r="B34" s="7"/>
       <c r="C34" s="12"/>
-      <c r="D34" s="16"/>
-    </row>
-    <row r="35" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D34" s="12"/>
+      <c r="E34" s="16"/>
+    </row>
+    <row r="35" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
       <c r="B35" s="9"/>
       <c r="C35" s="11"/>
-      <c r="D35" s="15"/>
-    </row>
-    <row r="36" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D35" s="11"/>
+      <c r="E35" s="15"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6"/>
       <c r="B36" s="7"/>
       <c r="C36" s="12"/>
-      <c r="D36" s="16"/>
-    </row>
-    <row r="37" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D36" s="12"/>
+      <c r="E36" s="16"/>
+    </row>
+    <row r="37" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8"/>
       <c r="B37" s="9"/>
       <c r="C37" s="11"/>
-      <c r="D37" s="15"/>
-    </row>
-    <row r="38" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D37" s="11"/>
+      <c r="E37" s="15"/>
+    </row>
+    <row r="38" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
       <c r="B38" s="7"/>
       <c r="C38" s="12"/>
-      <c r="D38" s="16"/>
-    </row>
-    <row r="39" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D38" s="12"/>
+      <c r="E38" s="16"/>
+    </row>
+    <row r="39" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" s="9"/>
       <c r="C39" s="11"/>
-      <c r="D39" s="15"/>
-    </row>
-    <row r="40" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D39" s="11"/>
+      <c r="E39" s="15"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6"/>
       <c r="B40" s="7"/>
       <c r="C40" s="12"/>
-      <c r="D40" s="16"/>
-    </row>
-    <row r="41" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D40" s="12"/>
+      <c r="E40" s="16"/>
+    </row>
+    <row r="41" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
       <c r="B41" s="9"/>
       <c r="C41" s="11"/>
-      <c r="D41" s="15"/>
-    </row>
-    <row r="42" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D41" s="11"/>
+      <c r="E41" s="15"/>
+    </row>
+    <row r="42" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6"/>
       <c r="B42" s="7"/>
       <c r="C42" s="12"/>
-      <c r="D42" s="16"/>
-    </row>
-    <row r="43" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D42" s="12"/>
+      <c r="E42" s="16"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
       <c r="B43" s="9"/>
       <c r="C43" s="11"/>
-      <c r="D43" s="15"/>
-    </row>
-    <row r="44" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D43" s="11"/>
+      <c r="E43" s="15"/>
+    </row>
+    <row r="44" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
       <c r="B44" s="7"/>
       <c r="C44" s="12"/>
-      <c r="D44" s="16"/>
-    </row>
-    <row r="45" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D44" s="12"/>
+      <c r="E44" s="16"/>
+    </row>
+    <row r="45" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
       <c r="B45" s="9"/>
       <c r="C45" s="11"/>
-      <c r="D45" s="15"/>
-    </row>
-    <row r="46" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D45" s="11"/>
+      <c r="E45" s="15"/>
+    </row>
+    <row r="46" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6"/>
       <c r="B46" s="7"/>
       <c r="C46" s="12"/>
-      <c r="D46" s="16"/>
-    </row>
-    <row r="47" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D46" s="12"/>
+      <c r="E46" s="16"/>
+    </row>
+    <row r="47" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8"/>
       <c r="B47" s="9"/>
       <c r="C47" s="11"/>
-      <c r="D47" s="15"/>
-    </row>
-    <row r="48" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D47" s="11"/>
+      <c r="E47" s="15"/>
+    </row>
+    <row r="48" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
       <c r="B48" s="7"/>
       <c r="C48" s="12"/>
-      <c r="D48" s="16"/>
-    </row>
-    <row r="49" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D48" s="12"/>
+      <c r="E48" s="16"/>
+    </row>
+    <row r="49" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8"/>
       <c r="B49" s="9"/>
       <c r="C49" s="11"/>
-      <c r="D49" s="15"/>
-    </row>
-    <row r="50" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D49" s="11"/>
+      <c r="E49" s="15"/>
+    </row>
+    <row r="50" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6"/>
       <c r="B50" s="7"/>
       <c r="C50" s="12"/>
-      <c r="D50" s="16"/>
-    </row>
-    <row r="51" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D50" s="12"/>
+      <c r="E50" s="16"/>
+    </row>
+    <row r="51" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
-      <c r="D51" s="17"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D1:D2"/>
+  <mergeCells count="2">
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
   </mergeCells>
@@ -1143,43 +1196,43 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{467F41B6-50A5-F34D-9811-537B9541F979}">
   <dimension ref="B2:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5" customWidth="1"/>
     <col min="2" max="2" width="67" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>4</v>
       </c>
@@ -1193,12 +1246,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4880C39C-0BD9-B447-909B-7F37D33CA805}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
@@ -1206,19 +1259,19 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="19"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="19"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1226,37 +1279,37 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: ajouter le champ financement et adapter les formulaires pour la gestion des lots mixtes en conventions foyer-résidence (#2158)
</commit_message>
<xml_diff>
--- a/static/files/foyer_residence_logements.xlsx
+++ b/static/files/foyer_residence_logements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nicolasoudard/workspace/beta.gouv.fr/apilos/static/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayoub.bouchachia\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FD775BD-7784-D74C-BFAA-AB9A8474BCD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C234B24-6EDA-400B-B94E-576E934924E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36340" yWindow="2120" windowWidth="27400" windowHeight="16440" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
+    <workbookView xWindow="2655" yWindow="2595" windowWidth="21600" windowHeight="11295" xr2:uid="{5E94D4F8-9F67-BB48-B84E-2D90FAF38DE8}"/>
   </bookViews>
   <sheets>
     <sheet name="Logements" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Ici quelques explications</t>
   </si>
@@ -113,6 +113,9 @@
   </si>
   <si>
     <t>T1 bis</t>
+  </si>
+  <si>
+    <t>Financement</t>
   </si>
 </sst>
 </file>
@@ -339,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -370,6 +373,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -475,7 +484,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office 2013 – 2022">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -771,354 +780,398 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08021C90-1ACF-2A4C-A1B0-58A48A8F7007}">
-  <dimension ref="A1:L51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.6640625" customWidth="1"/>
-    <col min="2" max="4" width="20.83203125" customWidth="1"/>
+    <col min="1" max="1" width="29.625" customWidth="1"/>
+    <col min="2" max="4" width="20.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="51.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="22" t="s">
+      <c r="E1" s="22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="34" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="23"/>
-    </row>
-    <row r="3" spans="1:12" ht="19" x14ac:dyDescent="0.25">
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="23"/>
+    </row>
+    <row r="3" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
       <c r="B3" s="9"/>
       <c r="C3" s="11"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="14" t="s">
+      <c r="D3" s="11"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="7"/>
       <c r="C4" s="12"/>
-      <c r="D4" s="16"/>
-      <c r="E4" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="16"/>
+      <c r="F4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8"/>
       <c r="B5" s="9"/>
       <c r="C5" s="11"/>
-      <c r="D5" s="15"/>
-    </row>
-    <row r="6" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="11"/>
+      <c r="E5" s="15"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="7"/>
       <c r="C6" s="12"/>
-      <c r="D6" s="16"/>
-    </row>
-    <row r="7" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="12"/>
+      <c r="E6" s="16"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8"/>
       <c r="B7" s="9"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="4"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="15"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="7"/>
       <c r="C8" s="12"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="4"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="16"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
-    </row>
-    <row r="9" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="11"/>
-      <c r="D9" s="15"/>
-    </row>
-    <row r="10" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="11"/>
+      <c r="E9" s="15"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="7"/>
       <c r="C10" s="12"/>
-      <c r="D10" s="16"/>
-    </row>
-    <row r="11" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="12"/>
+      <c r="E10" s="16"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8"/>
       <c r="B11" s="9"/>
       <c r="C11" s="11"/>
-      <c r="D11" s="15"/>
-    </row>
-    <row r="12" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D11" s="11"/>
+      <c r="E11" s="15"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6"/>
       <c r="B12" s="7"/>
       <c r="C12" s="12"/>
-      <c r="D12" s="16"/>
-    </row>
-    <row r="13" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D12" s="12"/>
+      <c r="E12" s="16"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
       <c r="B13" s="9"/>
       <c r="C13" s="11"/>
-      <c r="D13" s="15"/>
-    </row>
-    <row r="14" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D13" s="11"/>
+      <c r="E13" s="15"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6"/>
       <c r="B14" s="7"/>
       <c r="C14" s="12"/>
-      <c r="D14" s="16"/>
-    </row>
-    <row r="15" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D14" s="12"/>
+      <c r="E14" s="16"/>
+    </row>
+    <row r="15" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8"/>
       <c r="B15" s="9"/>
       <c r="C15" s="11"/>
-      <c r="D15" s="15"/>
-    </row>
-    <row r="16" spans="1:12" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D15" s="11"/>
+      <c r="E15" s="15"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6"/>
       <c r="B16" s="7"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="16"/>
-    </row>
-    <row r="17" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D16" s="12"/>
+      <c r="E16" s="16"/>
+    </row>
+    <row r="17" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
       <c r="B17" s="9"/>
       <c r="C17" s="11"/>
-      <c r="D17" s="15"/>
-    </row>
-    <row r="18" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D17" s="11"/>
+      <c r="E17" s="15"/>
+    </row>
+    <row r="18" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
       <c r="B18" s="7"/>
       <c r="C18" s="12"/>
-      <c r="D18" s="16"/>
-    </row>
-    <row r="19" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D18" s="12"/>
+      <c r="E18" s="16"/>
+    </row>
+    <row r="19" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8"/>
       <c r="B19" s="9"/>
       <c r="C19" s="11"/>
-      <c r="D19" s="15"/>
-    </row>
-    <row r="20" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D19" s="11"/>
+      <c r="E19" s="15"/>
+    </row>
+    <row r="20" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6"/>
       <c r="B20" s="7"/>
       <c r="C20" s="12"/>
-      <c r="D20" s="16"/>
-    </row>
-    <row r="21" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D20" s="12"/>
+      <c r="E20" s="16"/>
+    </row>
+    <row r="21" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8"/>
       <c r="B21" s="9"/>
       <c r="C21" s="11"/>
-      <c r="D21" s="15"/>
-    </row>
-    <row r="22" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D21" s="11"/>
+      <c r="E21" s="15"/>
+    </row>
+    <row r="22" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6"/>
       <c r="B22" s="7"/>
       <c r="C22" s="12"/>
-      <c r="D22" s="16"/>
-    </row>
-    <row r="23" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D22" s="12"/>
+      <c r="E22" s="16"/>
+    </row>
+    <row r="23" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8"/>
       <c r="B23" s="9"/>
       <c r="C23" s="11"/>
-      <c r="D23" s="15"/>
-    </row>
-    <row r="24" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D23" s="11"/>
+      <c r="E23" s="15"/>
+    </row>
+    <row r="24" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6"/>
       <c r="B24" s="7"/>
       <c r="C24" s="12"/>
-      <c r="D24" s="16"/>
-    </row>
-    <row r="25" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D24" s="12"/>
+      <c r="E24" s="16"/>
+    </row>
+    <row r="25" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="8"/>
       <c r="B25" s="9"/>
       <c r="C25" s="11"/>
-      <c r="D25" s="15"/>
-    </row>
-    <row r="26" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D25" s="11"/>
+      <c r="E25" s="15"/>
+    </row>
+    <row r="26" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6"/>
       <c r="B26" s="7"/>
       <c r="C26" s="12"/>
-      <c r="D26" s="16"/>
-    </row>
-    <row r="27" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D26" s="12"/>
+      <c r="E26" s="16"/>
+    </row>
+    <row r="27" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8"/>
       <c r="B27" s="9"/>
       <c r="C27" s="11"/>
-      <c r="D27" s="15"/>
-    </row>
-    <row r="28" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D27" s="11"/>
+      <c r="E27" s="15"/>
+    </row>
+    <row r="28" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="7"/>
       <c r="C28" s="12"/>
-      <c r="D28" s="16"/>
-    </row>
-    <row r="29" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D28" s="12"/>
+      <c r="E28" s="16"/>
+    </row>
+    <row r="29" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8"/>
       <c r="B29" s="9"/>
       <c r="C29" s="11"/>
-      <c r="D29" s="15"/>
-    </row>
-    <row r="30" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D29" s="11"/>
+      <c r="E29" s="15"/>
+    </row>
+    <row r="30" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6"/>
       <c r="B30" s="7"/>
       <c r="C30" s="12"/>
-      <c r="D30" s="16"/>
-    </row>
-    <row r="31" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D30" s="12"/>
+      <c r="E30" s="16"/>
+    </row>
+    <row r="31" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="8"/>
       <c r="B31" s="9"/>
       <c r="C31" s="11"/>
-      <c r="D31" s="15"/>
-    </row>
-    <row r="32" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D31" s="11"/>
+      <c r="E31" s="15"/>
+    </row>
+    <row r="32" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6"/>
       <c r="B32" s="7"/>
       <c r="C32" s="12"/>
-      <c r="D32" s="16"/>
-    </row>
-    <row r="33" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D32" s="12"/>
+      <c r="E32" s="16"/>
+    </row>
+    <row r="33" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
       <c r="B33" s="9"/>
       <c r="C33" s="11"/>
-      <c r="D33" s="15"/>
-    </row>
-    <row r="34" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D33" s="11"/>
+      <c r="E33" s="15"/>
+    </row>
+    <row r="34" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6"/>
       <c r="B34" s="7"/>
       <c r="C34" s="12"/>
-      <c r="D34" s="16"/>
-    </row>
-    <row r="35" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D34" s="12"/>
+      <c r="E34" s="16"/>
+    </row>
+    <row r="35" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="8"/>
       <c r="B35" s="9"/>
       <c r="C35" s="11"/>
-      <c r="D35" s="15"/>
-    </row>
-    <row r="36" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D35" s="11"/>
+      <c r="E35" s="15"/>
+    </row>
+    <row r="36" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6"/>
       <c r="B36" s="7"/>
       <c r="C36" s="12"/>
-      <c r="D36" s="16"/>
-    </row>
-    <row r="37" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D36" s="12"/>
+      <c r="E36" s="16"/>
+    </row>
+    <row r="37" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="8"/>
       <c r="B37" s="9"/>
       <c r="C37" s="11"/>
-      <c r="D37" s="15"/>
-    </row>
-    <row r="38" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D37" s="11"/>
+      <c r="E37" s="15"/>
+    </row>
+    <row r="38" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6"/>
       <c r="B38" s="7"/>
       <c r="C38" s="12"/>
-      <c r="D38" s="16"/>
-    </row>
-    <row r="39" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D38" s="12"/>
+      <c r="E38" s="16"/>
+    </row>
+    <row r="39" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="8"/>
       <c r="B39" s="9"/>
       <c r="C39" s="11"/>
-      <c r="D39" s="15"/>
-    </row>
-    <row r="40" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D39" s="11"/>
+      <c r="E39" s="15"/>
+    </row>
+    <row r="40" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6"/>
       <c r="B40" s="7"/>
       <c r="C40" s="12"/>
-      <c r="D40" s="16"/>
-    </row>
-    <row r="41" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D40" s="12"/>
+      <c r="E40" s="16"/>
+    </row>
+    <row r="41" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="8"/>
       <c r="B41" s="9"/>
       <c r="C41" s="11"/>
-      <c r="D41" s="15"/>
-    </row>
-    <row r="42" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D41" s="11"/>
+      <c r="E41" s="15"/>
+    </row>
+    <row r="42" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6"/>
       <c r="B42" s="7"/>
       <c r="C42" s="12"/>
-      <c r="D42" s="16"/>
-    </row>
-    <row r="43" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D42" s="12"/>
+      <c r="E42" s="16"/>
+    </row>
+    <row r="43" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="8"/>
       <c r="B43" s="9"/>
       <c r="C43" s="11"/>
-      <c r="D43" s="15"/>
-    </row>
-    <row r="44" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D43" s="11"/>
+      <c r="E43" s="15"/>
+    </row>
+    <row r="44" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="6"/>
       <c r="B44" s="7"/>
       <c r="C44" s="12"/>
-      <c r="D44" s="16"/>
-    </row>
-    <row r="45" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D44" s="12"/>
+      <c r="E44" s="16"/>
+    </row>
+    <row r="45" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
       <c r="B45" s="9"/>
       <c r="C45" s="11"/>
-      <c r="D45" s="15"/>
-    </row>
-    <row r="46" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D45" s="11"/>
+      <c r="E45" s="15"/>
+    </row>
+    <row r="46" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6"/>
       <c r="B46" s="7"/>
       <c r="C46" s="12"/>
-      <c r="D46" s="16"/>
-    </row>
-    <row r="47" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D46" s="12"/>
+      <c r="E46" s="16"/>
+    </row>
+    <row r="47" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="8"/>
       <c r="B47" s="9"/>
       <c r="C47" s="11"/>
-      <c r="D47" s="15"/>
-    </row>
-    <row r="48" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D47" s="11"/>
+      <c r="E47" s="15"/>
+    </row>
+    <row r="48" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6"/>
       <c r="B48" s="7"/>
       <c r="C48" s="12"/>
-      <c r="D48" s="16"/>
-    </row>
-    <row r="49" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D48" s="12"/>
+      <c r="E48" s="16"/>
+    </row>
+    <row r="49" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="8"/>
       <c r="B49" s="9"/>
       <c r="C49" s="11"/>
-      <c r="D49" s="15"/>
-    </row>
-    <row r="50" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D49" s="11"/>
+      <c r="E49" s="15"/>
+    </row>
+    <row r="50" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6"/>
       <c r="B50" s="7"/>
       <c r="C50" s="12"/>
-      <c r="D50" s="16"/>
-    </row>
-    <row r="51" spans="1:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D50" s="12"/>
+      <c r="E50" s="16"/>
+    </row>
+    <row r="51" spans="1:5" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5"/>
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
-      <c r="D51" s="17"/>
+      <c r="D51" s="13"/>
+      <c r="E51" s="17"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D1:D2"/>
+  <mergeCells count="2">
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:C2"/>
   </mergeCells>
@@ -1143,43 +1196,43 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{467F41B6-50A5-F34D-9811-537B9541F979}">
   <dimension ref="B2:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5" customWidth="1"/>
     <col min="2" max="2" width="67" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>4</v>
       </c>
@@ -1193,12 +1246,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4880C39C-0BD9-B447-909B-7F37D33CA805}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="42.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>6</v>
       </c>
@@ -1206,19 +1259,19 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="E2" s="19"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E3" s="19"/>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -1226,37 +1279,37 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="21"/>
     </row>
   </sheetData>

</xml_diff>